<commit_message>
Trazabilidad: días de stock en el semáforo y en todas las vistas
Días de stock = stock ÷ consumo por día (Stock_MP, col. G; en el PT, venta por día, Stock_PT col. F).
Se muestran en el semáforo (por código, con seguridad, punto de pedido y máximo en días, y el
código con menos días de cada almacén), en las tarjetas del kanban, el detalle de cada MP, los
lugares del almacén, la vista previa de la planilla, el semáforo y el kanban de PT y el dashboard.
La planilla de conteo suma «Consumo por día» y «Días de stock» (fórmula). Word actualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Planilla_conteo_MP.xlsx
+++ b/salida/Planilla_conteo_MP.xlsx
@@ -43,9 +43,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -152,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,6 +167,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -533,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -583,36 +585,43 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Solo se completan las celdas amarillas. «Estado» se calcula solo contra la seguridad y el punto de pedido.</t>
+          <t>Solo se completan las celdas amarillas. «Estado» se calcula solo contra la seguridad y el punto de pedido; «Días de</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cuándo se cuenta: en cada revisión periódica del proveedor (cada 10, 20 o 60 días hábiles según el código, Word de MP</t>
+          <t>stock» = stock contado ÷ consumo por día (Stock_MP, col. G: consumo del año ÷ 240 días hábiles).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Cuándo se cuenta: en cada revisión periódica del proveedor (cada 10, 20 o 60 días hábiles según el código, Word de MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>sección 9) y siempre que un retiro deje una tarjeta cerca del punto de pedido.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Fuentes: MP-FLAMA2035.xlsx › Stock_MP (L seguridad, K consumo mientras llega, S máximo, U lugares) y Almacenes (lugares).</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Fuentes: MP-FLAMA2035.xlsx › Stock_MP (L seguridad, K consumo mientras llega, S máximo, U lugares) y Almacenes (lugares).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Punto de pedido = L + K. Lugar de cada código: criterio de reparto explicado en el Word de trazabilidad (sección 3).</t>
         </is>
@@ -629,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -640,9 +649,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -717,15 +728,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -766,12 +787,19 @@
       <c r="H6" s="10" t="n">
         <v>922.5</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>24.9585</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -808,12 +836,19 @@
       <c r="H7" s="10" t="n">
         <v>3007.6</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>94.82089999999999</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -850,12 +885,19 @@
       <c r="H8" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>0.6943</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -892,12 +934,19 @@
       <c r="H9" s="10" t="n">
         <v>10.2</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>0.1134</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -934,12 +983,19 @@
       <c r="H10" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>0.4156</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -976,12 +1032,19 @@
       <c r="H11" s="10" t="n">
         <v>10.1</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>0.0945</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1018,12 +1081,19 @@
       <c r="H12" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>0.0756</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1060,19 +1130,26 @@
       <c r="H13" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>0.0324</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1087,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1098,9 +1175,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1175,15 +1254,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1224,12 +1313,19 @@
       <c r="H6" s="10" t="n">
         <v>233.7</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>33.1652</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1266,12 +1362,19 @@
       <c r="H7" s="10" t="n">
         <v>113.4</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>15.2178</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1308,12 +1411,19 @@
       <c r="H8" s="10" t="n">
         <v>77.3</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>10.2709</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1350,19 +1460,26 @@
       <c r="H9" s="10" t="n">
         <v>21.3</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>3.3356</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1377,7 +1494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1388,9 +1505,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1465,15 +1584,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1514,12 +1643,19 @@
       <c r="H6" s="10" t="n">
         <v>399.3</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>6.4776</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1556,12 +1692,19 @@
       <c r="H7" s="10" t="n">
         <v>606.3</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>14.237</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1598,12 +1741,19 @@
       <c r="H8" s="10" t="n">
         <v>147.4</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>5.1798</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1640,12 +1790,19 @@
       <c r="H9" s="10" t="n">
         <v>344.7</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>10.3573</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1682,19 +1839,26 @@
       <c r="H10" s="10" t="n">
         <v>91.2</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>2.5899</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1709,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1720,9 +1884,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1797,15 +1963,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1846,12 +2022,19 @@
       <c r="H6" s="10" t="n">
         <v>149.3</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>3.7806</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1888,12 +2071,19 @@
       <c r="H7" s="10" t="n">
         <v>227.6</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>8.316599999999999</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1930,12 +2120,19 @@
       <c r="H8" s="10" t="n">
         <v>98.59999999999999</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>4.1583</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1972,12 +2169,19 @@
       <c r="H9" s="10" t="n">
         <v>21.2</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -2014,12 +2218,19 @@
       <c r="H10" s="10" t="n">
         <v>53.9</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>1.8903</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2056,12 +2267,19 @@
       <c r="H11" s="10" t="n">
         <v>141.7</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>5.6709</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2098,12 +2316,19 @@
       <c r="H12" s="10" t="n">
         <v>102.1</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>1.5126</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -2140,12 +2365,19 @@
       <c r="H13" s="10" t="n">
         <v>1042.3</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>30.2447</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2182,12 +2414,19 @@
       <c r="H14" s="10" t="n">
         <v>63.9</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>1.8903</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -2224,12 +2463,19 @@
       <c r="H15" s="10" t="n">
         <v>108.6</v>
       </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="12">
-        <f>IF(I15="","",IF(I15&lt;=F15,"BAJO SEGURIDAD",IF(I15&lt;=G15,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K15" s="9" t="n"/>
+      <c r="I15" s="11" t="n">
+        <v>4.1583</v>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="10">
+        <f>IFERROR(IF(OR(J15="",I15=0),"",J15/I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(J15="","",IF(J15&lt;=F15,"BAJO SEGURIDAD",IF(J15&lt;=G15,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -2266,12 +2512,19 @@
       <c r="H16" s="10" t="n">
         <v>53.9</v>
       </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12">
-        <f>IF(I16="","",IF(I16&lt;=F16,"BAJO SEGURIDAD",IF(I16&lt;=G16,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K16" s="9" t="n"/>
+      <c r="I16" s="11" t="n">
+        <v>1.8903</v>
+      </c>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="10">
+        <f>IFERROR(IF(OR(J16="",I16=0),"",J16/I16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="13">
+        <f>IF(J16="","",IF(J16&lt;=F16,"BAJO SEGURIDAD",IF(J16&lt;=G16,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -2308,12 +2561,19 @@
       <c r="H17" s="10" t="n">
         <v>76.2</v>
       </c>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="12">
-        <f>IF(I17="","",IF(I17&lt;=F17,"BAJO SEGURIDAD",IF(I17&lt;=G17,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K17" s="9" t="n"/>
+      <c r="I17" s="11" t="n">
+        <v>3.0251</v>
+      </c>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="10">
+        <f>IFERROR(IF(OR(J17="",I17=0),"",J17/I17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="13">
+        <f>IF(J17="","",IF(J17&lt;=F17,"BAJO SEGURIDAD",IF(J17&lt;=G17,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -2350,12 +2610,19 @@
       <c r="H18" s="10" t="n">
         <v>140.2</v>
       </c>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="12">
-        <f>IF(I18="","",IF(I18&lt;=F18,"BAJO SEGURIDAD",IF(I18&lt;=G18,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K18" s="9" t="n"/>
+      <c r="I18" s="11" t="n">
+        <v>5.7942</v>
+      </c>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="10">
+        <f>IFERROR(IF(OR(J18="",I18=0),"",J18/I18),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="13">
+        <f>IF(J18="","",IF(J18&lt;=F18,"BAJO SEGURIDAD",IF(J18&lt;=G18,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2392,12 +2659,19 @@
       <c r="H19" s="10" t="n">
         <v>21.9</v>
       </c>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="12">
-        <f>IF(I19="","",IF(I19&lt;=F19,"BAJO SEGURIDAD",IF(I19&lt;=G19,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K19" s="9" t="n"/>
+      <c r="I19" s="11" t="n">
+        <v>0.9075</v>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="10">
+        <f>IFERROR(IF(OR(J19="",I19=0),"",J19/I19),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19="","",IF(J19&lt;=F19,"BAJO SEGURIDAD",IF(J19&lt;=G19,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -2434,12 +2708,19 @@
       <c r="H20" s="10" t="n">
         <v>21.9</v>
       </c>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="12">
-        <f>IF(I20="","",IF(I20&lt;=F20,"BAJO SEGURIDAD",IF(I20&lt;=G20,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K20" s="9" t="n"/>
+      <c r="I20" s="11" t="n">
+        <v>0.9075</v>
+      </c>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="10">
+        <f>IFERROR(IF(OR(J20="",I20=0),"",J20/I20),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="13">
+        <f>IF(J20="","",IF(J20&lt;=F20,"BAJO SEGURIDAD",IF(J20&lt;=G20,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -2476,12 +2757,19 @@
       <c r="H21" s="10" t="n">
         <v>1021.2</v>
       </c>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="12">
-        <f>IF(I21="","",IF(I21&lt;=F21,"BAJO SEGURIDAD",IF(I21&lt;=G21,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K21" s="9" t="n"/>
+      <c r="I21" s="11" t="n">
+        <v>15.1224</v>
+      </c>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="10">
+        <f>IFERROR(IF(OR(J21="",I21=0),"",J21/I21),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="13">
+        <f>IF(J21="","",IF(J21&lt;=F21,"BAJO SEGURIDAD",IF(J21&lt;=G21,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -2518,19 +2806,26 @@
       <c r="H22" s="10" t="n">
         <v>21.2</v>
       </c>
-      <c r="I22" s="11" t="n"/>
-      <c r="J22" s="12">
-        <f>IF(I22="","",IF(I22&lt;=F22,"BAJO SEGURIDAD",IF(I22&lt;=G22,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K22" s="9" t="n"/>
+      <c r="I22" s="11" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="10">
+        <f>IFERROR(IF(OR(J22="",I22=0),"",J22/I22),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="13">
+        <f>IF(J22="","",IF(J22&lt;=F22,"BAJO SEGURIDAD",IF(J22&lt;=G22,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M22" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2545,7 +2840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2556,9 +2851,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2633,15 +2930,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -2682,12 +2989,19 @@
       <c r="H6" s="10" t="n">
         <v>371.4</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>12.1176</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -2724,12 +3038,19 @@
       <c r="H7" s="10" t="n">
         <v>189.8</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>6.8778</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -2766,12 +3087,19 @@
       <c r="H8" s="10" t="n">
         <v>894.8</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>29.1887</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -2808,12 +3136,19 @@
       <c r="H9" s="10" t="n">
         <v>433.9</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>15.7356</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -2850,12 +3185,19 @@
       <c r="H10" s="10" t="n">
         <v>42.4</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>1.734</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2892,12 +3234,19 @@
       <c r="H11" s="10" t="n">
         <v>35.9</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>1.156</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2934,12 +3283,19 @@
       <c r="H12" s="10" t="n">
         <v>124.2</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>4.0469</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -2976,12 +3332,19 @@
       <c r="H13" s="10" t="n">
         <v>35.9</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>1.1571</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -3018,19 +3381,26 @@
       <c r="H14" s="10" t="n">
         <v>85.5</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>3.1006</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3045,7 +3415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3056,9 +3426,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3133,15 +3505,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -3182,12 +3564,19 @@
       <c r="H6" s="10" t="n">
         <v>441</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>18.7612</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -3224,12 +3613,19 @@
       <c r="H7" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -3266,12 +3662,19 @@
       <c r="H8" s="10" t="n">
         <v>552</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>22.1711</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -3308,12 +3711,19 @@
       <c r="H9" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>1.073</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -3350,12 +3760,19 @@
       <c r="H10" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>1.4563</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -3392,19 +3809,26 @@
       <c r="H11" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>0.6901</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3419,7 +3843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3430,9 +3854,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3507,15 +3933,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -3556,12 +3992,19 @@
       <c r="H6" s="10" t="n">
         <v>1306.3</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>50.3972</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -3598,12 +4041,19 @@
       <c r="H7" s="10" t="n">
         <v>1514.7</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>58.4358</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -3640,12 +4090,19 @@
       <c r="H8" s="10" t="n">
         <v>515.1</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>14.9043</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -3682,12 +4139,19 @@
       <c r="H9" s="10" t="n">
         <v>417.4</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>12.0763</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -3724,12 +4188,19 @@
       <c r="H10" s="10" t="n">
         <v>3544.5</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>136.7462</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -3766,12 +4237,19 @@
       <c r="H11" s="10" t="n">
         <v>2659.3</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>102.5971</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -3808,12 +4286,19 @@
       <c r="H12" s="10" t="n">
         <v>490</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>14.1796</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -3850,19 +4335,26 @@
       <c r="H13" s="10" t="n">
         <v>358.1</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>10.3607</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3877,7 +4369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3888,9 +4380,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3965,15 +4459,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -4014,12 +4518,19 @@
       <c r="H6" s="10" t="n">
         <v>46.9</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>2.1258</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -4056,12 +4567,19 @@
       <c r="H7" s="10" t="n">
         <v>12.7</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>0.5293</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -4098,12 +4616,19 @@
       <c r="H8" s="10" t="n">
         <v>9.1</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>0.3734</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -4140,19 +4665,26 @@
       <c r="H9" s="10" t="n">
         <v>6.3</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>0.2363</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4167,7 +4699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4178,9 +4710,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4255,15 +4789,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -4304,12 +4848,19 @@
       <c r="H6" s="10" t="n">
         <v>10207.5</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>1134.909</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -4346,12 +4897,19 @@
       <c r="H7" s="10" t="n">
         <v>4207.4</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>427.2206</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -4388,12 +4946,19 @@
       <c r="H8" s="10" t="n">
         <v>326.2</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>14.9247</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -4430,12 +4995,19 @@
       <c r="H9" s="10" t="n">
         <v>83.59999999999999</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>3.0333</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -4472,19 +5044,26 @@
       <c r="H10" s="10" t="n">
         <v>138.8</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4499,7 +5078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4510,9 +5089,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4587,15 +5168,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -4636,12 +5227,19 @@
       <c r="H6" s="10" t="n">
         <v>7923.7</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>844.2527</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -4678,12 +5276,19 @@
       <c r="H7" s="10" t="n">
         <v>817.8</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>58.8597</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -4720,12 +5325,19 @@
       <c r="H8" s="10" t="n">
         <v>2784.4</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>266.0527</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -4762,12 +5374,19 @@
       <c r="H9" s="10" t="n">
         <v>659.6</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>16.0955</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -4804,12 +5423,19 @@
       <c r="H10" s="10" t="n">
         <v>29034.3</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>1185.2607</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -4846,12 +5472,19 @@
       <c r="H11" s="10" t="n">
         <v>52.9</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>6.3863</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -4888,12 +5521,19 @@
       <c r="H12" s="10" t="n">
         <v>5766.5</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>178.2485</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -4930,12 +5570,19 @@
       <c r="H13" s="10" t="n">
         <v>23055.7</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>710.6167</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -4972,12 +5619,19 @@
       <c r="H14" s="10" t="n">
         <v>254.6</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>1.0773</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -5014,19 +5668,26 @@
       <c r="H15" s="10" t="n">
         <v>1016.3</v>
       </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="12">
-        <f>IF(I15="","",IF(I15&lt;=F15,"BAJO SEGURIDAD",IF(I15&lt;=G15,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K15" s="9" t="n"/>
+      <c r="I15" s="11" t="n">
+        <v>6.3863</v>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="10">
+        <f>IFERROR(IF(OR(J15="",I15=0),"",J15/I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(J15="","",IF(J15&lt;=F15,"BAJO SEGURIDAD",IF(J15&lt;=G15,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M15" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5041,7 +5702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5052,9 +5713,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5129,15 +5792,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -5178,12 +5851,19 @@
       <c r="H6" s="10" t="n">
         <v>22278.3</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>889.9425</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -5220,12 +5900,19 @@
       <c r="H7" s="10" t="n">
         <v>23472.1</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>885.1376</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -5262,12 +5949,19 @@
       <c r="H8" s="10" t="n">
         <v>3342.1</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>133.636</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -5304,12 +5998,19 @@
       <c r="H9" s="10" t="n">
         <v>1079.3</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>30.9852</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -5346,12 +6047,19 @@
       <c r="H10" s="10" t="n">
         <v>501.2</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>1.8903</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -5388,12 +6096,19 @@
       <c r="H11" s="10" t="n">
         <v>7517.9</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>308.2654</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -5430,12 +6145,19 @@
       <c r="H12" s="10" t="n">
         <v>1005.1</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>7.6872</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -5472,12 +6194,19 @@
       <c r="H13" s="10" t="n">
         <v>5518.8</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>235.4484</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -5514,12 +6243,19 @@
       <c r="H14" s="10" t="n">
         <v>7789.2</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>308.2654</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -5556,12 +6292,19 @@
       <c r="H15" s="10" t="n">
         <v>3328.7</v>
       </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="12">
-        <f>IF(I15="","",IF(I15&lt;=F15,"BAJO SEGURIDAD",IF(I15&lt;=G15,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K15" s="9" t="n"/>
+      <c r="I15" s="11" t="n">
+        <v>128.3957</v>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="10">
+        <f>IFERROR(IF(OR(J15="",I15=0),"",J15/I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(J15="","",IF(J15&lt;=F15,"BAJO SEGURIDAD",IF(J15&lt;=G15,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -5598,12 +6341,19 @@
       <c r="H16" s="10" t="n">
         <v>1002.7</v>
       </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12">
-        <f>IF(I16="","",IF(I16&lt;=F16,"BAJO SEGURIDAD",IF(I16&lt;=G16,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K16" s="9" t="n"/>
+      <c r="I16" s="11" t="n">
+        <v>4.1583</v>
+      </c>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="10">
+        <f>IFERROR(IF(OR(J16="",I16=0),"",J16/I16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="13">
+        <f>IF(J16="","",IF(J16&lt;=F16,"BAJO SEGURIDAD",IF(J16&lt;=G16,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -5640,12 +6390,19 @@
       <c r="H17" s="10" t="n">
         <v>250.6</v>
       </c>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="12">
-        <f>IF(I17="","",IF(I17&lt;=F17,"BAJO SEGURIDAD",IF(I17&lt;=G17,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K17" s="9" t="n"/>
+      <c r="I17" s="11" t="n">
+        <v>0.9075</v>
+      </c>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="10">
+        <f>IFERROR(IF(OR(J17="",I17=0),"",J17/I17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="13">
+        <f>IF(J17="","",IF(J17&lt;=F17,"BAJO SEGURIDAD",IF(J17&lt;=G17,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -5682,12 +6439,19 @@
       <c r="H18" s="10" t="n">
         <v>7789.2</v>
       </c>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="12">
-        <f>IF(I18="","",IF(I18&lt;=F18,"BAJO SEGURIDAD",IF(I18&lt;=G18,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K18" s="9" t="n"/>
+      <c r="I18" s="11" t="n">
+        <v>308.2654</v>
+      </c>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="10">
+        <f>IFERROR(IF(OR(J18="",I18=0),"",J18/I18),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="13">
+        <f>IF(J18="","",IF(J18&lt;=F18,"BAJO SEGURIDAD",IF(J18&lt;=G18,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -5724,12 +6488,19 @@
       <c r="H19" s="10" t="n">
         <v>7431.6</v>
       </c>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="12">
-        <f>IF(I19="","",IF(I19&lt;=F19,"BAJO SEGURIDAD",IF(I19&lt;=G19,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K19" s="9" t="n"/>
+      <c r="I19" s="11" t="n">
+        <v>308.2654</v>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="10">
+        <f>IFERROR(IF(OR(J19="",I19=0),"",J19/I19),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19="","",IF(J19&lt;=F19,"BAJO SEGURIDAD",IF(J19&lt;=G19,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -5766,12 +6537,19 @@
       <c r="H20" s="10" t="n">
         <v>250.4</v>
       </c>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="12">
-        <f>IF(I20="","",IF(I20&lt;=F20,"BAJO SEGURIDAD",IF(I20&lt;=G20,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K20" s="9" t="n"/>
+      <c r="I20" s="11" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="10">
+        <f>IFERROR(IF(OR(J20="",I20=0),"",J20/I20),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="13">
+        <f>IF(J20="","",IF(J20&lt;=F20,"BAJO SEGURIDAD",IF(J20&lt;=G20,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -5808,19 +6586,26 @@
       <c r="H21" s="10" t="n">
         <v>3512.2</v>
       </c>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="12">
-        <f>IF(I21="","",IF(I21&lt;=F21,"BAJO SEGURIDAD",IF(I21&lt;=G21,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K21" s="9" t="n"/>
+      <c r="I21" s="11" t="n">
+        <v>152.3182</v>
+      </c>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="10">
+        <f>IFERROR(IF(OR(J21="",I21=0),"",J21/I21),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="13">
+        <f>IF(J21="","",IF(J21&lt;=F21,"BAJO SEGURIDAD",IF(J21&lt;=G21,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M21" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5835,7 +6620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5846,9 +6631,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5923,15 +6710,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -5972,12 +6769,19 @@
       <c r="H6" s="10" t="n">
         <v>22147.2</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>844.2527</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -6014,12 +6818,19 @@
       <c r="H7" s="10" t="n">
         <v>8973.200000000001</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>341.008</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -6056,12 +6867,19 @@
       <c r="H8" s="10" t="n">
         <v>3275.3</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>133.636</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -6098,12 +6916,19 @@
       <c r="H9" s="10" t="n">
         <v>4844.2</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>167.0682</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -6140,12 +6965,19 @@
       <c r="H10" s="10" t="n">
         <v>7335</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>308.2654</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -6182,12 +7014,19 @@
       <c r="H11" s="10" t="n">
         <v>3175.3</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>133.636</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -6224,12 +7063,19 @@
       <c r="H12" s="10" t="n">
         <v>3064.5</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>128.3957</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -6266,12 +7112,19 @@
       <c r="H13" s="10" t="n">
         <v>3128.7</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>128.3957</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -6308,12 +7161,19 @@
       <c r="H14" s="10" t="n">
         <v>3242.1</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>133.636</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -6350,12 +7210,19 @@
       <c r="H15" s="10" t="n">
         <v>863.8</v>
       </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="12">
-        <f>IF(I15="","",IF(I15&lt;=F15,"BAJO SEGURIDAD",IF(I15&lt;=G15,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K15" s="9" t="n"/>
+      <c r="I15" s="11" t="n">
+        <v>30.9852</v>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="10">
+        <f>IFERROR(IF(OR(J15="",I15=0),"",J15/I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(J15="","",IF(J15&lt;=F15,"BAJO SEGURIDAD",IF(J15&lt;=G15,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -6392,12 +7259,19 @@
       <c r="H16" s="10" t="n">
         <v>3064.5</v>
       </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12">
-        <f>IF(I16="","",IF(I16&lt;=F16,"BAJO SEGURIDAD",IF(I16&lt;=G16,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K16" s="9" t="n"/>
+      <c r="I16" s="11" t="n">
+        <v>128.3957</v>
+      </c>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="10">
+        <f>IFERROR(IF(OR(J16="",I16=0),"",J16/I16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="13">
+        <f>IF(J16="","",IF(J16&lt;=F16,"BAJO SEGURIDAD",IF(J16&lt;=G16,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -6434,12 +7308,19 @@
       <c r="H17" s="10" t="n">
         <v>763.8</v>
       </c>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="12">
-        <f>IF(I17="","",IF(I17&lt;=F17,"BAJO SEGURIDAD",IF(I17&lt;=G17,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K17" s="9" t="n"/>
+      <c r="I17" s="11" t="n">
+        <v>30.9852</v>
+      </c>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="10">
+        <f>IFERROR(IF(OR(J17="",I17=0),"",J17/I17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="13">
+        <f>IF(J17="","",IF(J17&lt;=F17,"BAJO SEGURIDAD",IF(J17&lt;=G17,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -6476,12 +7357,19 @@
       <c r="H18" s="10" t="n">
         <v>8467.799999999999</v>
       </c>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="12">
-        <f>IF(I18="","",IF(I18&lt;=F18,"BAJO SEGURIDAD",IF(I18&lt;=G18,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K18" s="9" t="n"/>
+      <c r="I18" s="11" t="n">
+        <v>334.1364</v>
+      </c>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="10">
+        <f>IFERROR(IF(OR(J18="",I18=0),"",J18/I18),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="13">
+        <f>IF(J18="","",IF(J18&lt;=F18,"BAJO SEGURIDAD",IF(J18&lt;=G18,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -6518,12 +7406,19 @@
       <c r="H19" s="10" t="n">
         <v>3187.1</v>
       </c>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="12">
-        <f>IF(I19="","",IF(I19&lt;=F19,"BAJO SEGURIDAD",IF(I19&lt;=G19,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K19" s="9" t="n"/>
+      <c r="I19" s="11" t="n">
+        <v>133.636</v>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="10">
+        <f>IFERROR(IF(OR(J19="",I19=0),"",J19/I19),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19="","",IF(J19&lt;=F19,"BAJO SEGURIDAD",IF(J19&lt;=G19,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -6560,12 +7455,19 @@
       <c r="H20" s="10" t="n">
         <v>4242.4</v>
       </c>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="12">
-        <f>IF(I20="","",IF(I20&lt;=F20,"BAJO SEGURIDAD",IF(I20&lt;=G20,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K20" s="9" t="n"/>
+      <c r="I20" s="11" t="n">
+        <v>173.1168</v>
+      </c>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="10">
+        <f>IFERROR(IF(OR(J20="",I20=0),"",J20/I20),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="13">
+        <f>IF(J20="","",IF(J20&lt;=F20,"BAJO SEGURIDAD",IF(J20&lt;=G20,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -6602,12 +7504,19 @@
       <c r="H21" s="10" t="n">
         <v>779.3</v>
       </c>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="12">
-        <f>IF(I21="","",IF(I21&lt;=F21,"BAJO SEGURIDAD",IF(I21&lt;=G21,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K21" s="9" t="n"/>
+      <c r="I21" s="11" t="n">
+        <v>30.9852</v>
+      </c>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="10">
+        <f>IFERROR(IF(OR(J21="",I21=0),"",J21/I21),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="13">
+        <f>IF(J21="","",IF(J21&lt;=F21,"BAJO SEGURIDAD",IF(J21&lt;=G21,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -6644,12 +7553,19 @@
       <c r="H22" s="10" t="n">
         <v>215.8</v>
       </c>
-      <c r="I22" s="11" t="n"/>
-      <c r="J22" s="12">
-        <f>IF(I22="","",IF(I22&lt;=F22,"BAJO SEGURIDAD",IF(I22&lt;=G22,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K22" s="9" t="n"/>
+      <c r="I22" s="11" t="n">
+        <v>7.6872</v>
+      </c>
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="10">
+        <f>IFERROR(IF(OR(J22="",I22=0),"",J22/I22),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="13">
+        <f>IF(J22="","",IF(J22&lt;=F22,"BAJO SEGURIDAD",IF(J22&lt;=G22,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -6686,12 +7602,19 @@
       <c r="H23" s="10" t="n">
         <v>215.8</v>
       </c>
-      <c r="I23" s="11" t="n"/>
-      <c r="J23" s="12">
-        <f>IF(I23="","",IF(I23&lt;=F23,"BAJO SEGURIDAD",IF(I23&lt;=G23,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K23" s="9" t="n"/>
+      <c r="I23" s="11" t="n">
+        <v>7.6872</v>
+      </c>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="10">
+        <f>IFERROR(IF(OR(J23="",I23=0),"",J23/I23),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="13">
+        <f>IF(J23="","",IF(J23&lt;=F23,"BAJO SEGURIDAD",IF(J23&lt;=G23,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -6728,19 +7651,26 @@
       <c r="H24" s="10" t="n">
         <v>219.7</v>
       </c>
-      <c r="I24" s="11" t="n"/>
-      <c r="J24" s="12">
-        <f>IF(I24="","",IF(I24&lt;=F24,"BAJO SEGURIDAD",IF(I24&lt;=G24,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K24" s="9" t="n"/>
+      <c r="I24" s="11" t="n">
+        <v>7.6872</v>
+      </c>
+      <c r="J24" s="12" t="n"/>
+      <c r="K24" s="10">
+        <f>IFERROR(IF(OR(J24="",I24=0),"",J24/I24),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="13">
+        <f>IF(J24="","",IF(J24&lt;=F24,"BAJO SEGURIDAD",IF(J24&lt;=G24,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M24" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -6755,7 +7685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6766,9 +7696,11 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6843,15 +7775,25 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
+          <t>Consumo por día</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
           <t>Stock contado</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Días de stock</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -6892,12 +7834,19 @@
       <c r="H6" s="10" t="n">
         <v>52.2</v>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12">
-        <f>IF(I6="","",IF(I6&lt;=F6,"BAJO SEGURIDAD",IF(I6&lt;=G6,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>0.7763</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="10">
+        <f>IFERROR(IF(OR(J6="",I6=0),"",J6/I6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(J6="","",IF(J6&lt;=F6,"BAJO SEGURIDAD",IF(J6&lt;=G6,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -6934,12 +7883,19 @@
       <c r="H7" s="10" t="n">
         <v>60.5</v>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12">
-        <f>IF(I7="","",IF(I7&lt;=F7,"BAJO SEGURIDAD",IF(I7&lt;=G7,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K7" s="9" t="n"/>
+      <c r="I7" s="11" t="n">
+        <v>2.111</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="10">
+        <f>IFERROR(IF(OR(J7="",I7=0),"",J7/I7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(J7="","",IF(J7&lt;=F7,"BAJO SEGURIDAD",IF(J7&lt;=G7,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -6976,12 +7932,19 @@
       <c r="H8" s="10" t="n">
         <v>887.4</v>
       </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="12">
-        <f>IF(I8="","",IF(I8&lt;=F8,"BAJO SEGURIDAD",IF(I8&lt;=G8,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="I8" s="11" t="n">
+        <v>30.9129</v>
+      </c>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="10">
+        <f>IFERROR(IF(OR(J8="",I8=0),"",J8/I8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(J8="","",IF(J8&lt;=F8,"BAJO SEGURIDAD",IF(J8&lt;=G8,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -7018,12 +7981,19 @@
       <c r="H9" s="10" t="n">
         <v>11893.7</v>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12">
-        <f>IF(I9="","",IF(I9&lt;=F9,"BAJO SEGURIDAD",IF(I9&lt;=G9,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K9" s="9" t="n"/>
+      <c r="I9" s="11" t="n">
+        <v>424.5315</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="10">
+        <f>IFERROR(IF(OR(J9="",I9=0),"",J9/I9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(J9="","",IF(J9&lt;=F9,"BAJO SEGURIDAD",IF(J9&lt;=G9,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -7060,12 +8030,19 @@
       <c r="H10" s="10" t="n">
         <v>439.6</v>
       </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="12">
-        <f>IF(I10="","",IF(I10&lt;=F10,"BAJO SEGURIDAD",IF(I10&lt;=G10,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="I10" s="11" t="n">
+        <v>13.0074</v>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="10">
+        <f>IFERROR(IF(OR(J10="",I10=0),"",J10/I10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(J10="","",IF(J10&lt;=F10,"BAJO SEGURIDAD",IF(J10&lt;=G10,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -7102,12 +8079,19 @@
       <c r="H11" s="10" t="n">
         <v>12595.2</v>
       </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="12">
-        <f>IF(I11="","",IF(I11&lt;=F11,"BAJO SEGURIDAD",IF(I11&lt;=G11,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K11" s="9" t="n"/>
+      <c r="I11" s="11" t="n">
+        <v>449.6974</v>
+      </c>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="10">
+        <f>IFERROR(IF(OR(J11="",I11=0),"",J11/I11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(J11="","",IF(J11&lt;=F11,"BAJO SEGURIDAD",IF(J11&lt;=G11,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -7144,12 +8128,19 @@
       <c r="H12" s="10" t="n">
         <v>11946.7</v>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12">
-        <f>IF(I12="","",IF(I12&lt;=F12,"BAJO SEGURIDAD",IF(I12&lt;=G12,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K12" s="9" t="n"/>
+      <c r="I12" s="11" t="n">
+        <v>449.6974</v>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="10">
+        <f>IFERROR(IF(OR(J12="",I12=0),"",J12/I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(J12="","",IF(J12&lt;=F12,"BAJO SEGURIDAD",IF(J12&lt;=G12,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -7186,12 +8177,19 @@
       <c r="H13" s="10" t="n">
         <v>12595.2</v>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12">
-        <f>IF(I13="","",IF(I13&lt;=F13,"BAJO SEGURIDAD",IF(I13&lt;=G13,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K13" s="9" t="n"/>
+      <c r="I13" s="11" t="n">
+        <v>449.6974</v>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="10">
+        <f>IFERROR(IF(OR(J13="",I13=0),"",J13/I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(J13="","",IF(J13&lt;=F13,"BAJO SEGURIDAD",IF(J13&lt;=G13,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -7228,12 +8226,19 @@
       <c r="H14" s="10" t="n">
         <v>9078.799999999999</v>
       </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="12">
-        <f>IF(I14="","",IF(I14&lt;=F14,"BAJO SEGURIDAD",IF(I14&lt;=G14,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K14" s="9" t="n"/>
+      <c r="I14" s="11" t="n">
+        <v>356.3724</v>
+      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="10">
+        <f>IFERROR(IF(OR(J14="",I14=0),"",J14/I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(J14="","",IF(J14&lt;=F14,"BAJO SEGURIDAD",IF(J14&lt;=G14,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -7270,12 +8275,19 @@
       <c r="H15" s="10" t="n">
         <v>9078.799999999999</v>
       </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="12">
-        <f>IF(I15="","",IF(I15&lt;=F15,"BAJO SEGURIDAD",IF(I15&lt;=G15,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K15" s="9" t="n"/>
+      <c r="I15" s="11" t="n">
+        <v>356.3724</v>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="10">
+        <f>IFERROR(IF(OR(J15="",I15=0),"",J15/I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(J15="","",IF(J15&lt;=F15,"BAJO SEGURIDAD",IF(J15&lt;=G15,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -7312,12 +8324,19 @@
       <c r="H16" s="10" t="n">
         <v>102.1</v>
       </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12">
-        <f>IF(I16="","",IF(I16&lt;=F16,"BAJO SEGURIDAD",IF(I16&lt;=G16,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K16" s="9" t="n"/>
+      <c r="I16" s="11" t="n">
+        <v>0.5810999999999999</v>
+      </c>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="10">
+        <f>IFERROR(IF(OR(J16="",I16=0),"",J16/I16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="13">
+        <f>IF(J16="","",IF(J16&lt;=F16,"BAJO SEGURIDAD",IF(J16&lt;=G16,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -7354,12 +8373,19 @@
       <c r="H17" s="10" t="n">
         <v>100.1</v>
       </c>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="12">
-        <f>IF(I17="","",IF(I17&lt;=F17,"BAJO SEGURIDAD",IF(I17&lt;=G17,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K17" s="9" t="n"/>
+      <c r="I17" s="11" t="n">
+        <v>0.4605</v>
+      </c>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="10">
+        <f>IFERROR(IF(OR(J17="",I17=0),"",J17/I17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="13">
+        <f>IF(J17="","",IF(J17&lt;=F17,"BAJO SEGURIDAD",IF(J17&lt;=G17,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -7396,12 +8422,19 @@
       <c r="H18" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="12">
-        <f>IF(I18="","",IF(I18&lt;=F18,"BAJO SEGURIDAD",IF(I18&lt;=G18,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K18" s="9" t="n"/>
+      <c r="I18" s="11" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="10">
+        <f>IFERROR(IF(OR(J18="",I18=0),"",J18/I18),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="13">
+        <f>IF(J18="","",IF(J18&lt;=F18,"BAJO SEGURIDAD",IF(J18&lt;=G18,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -7438,19 +8471,26 @@
       <c r="H19" s="10" t="n">
         <v>39.2</v>
       </c>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="12">
-        <f>IF(I19="","",IF(I19&lt;=F19,"BAJO SEGURIDAD",IF(I19&lt;=G19,"PEDIR","OK")))</f>
-        <v/>
-      </c>
-      <c r="K19" s="9" t="n"/>
+      <c r="I19" s="11" t="n">
+        <v>1.1533</v>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="10">
+        <f>IFERROR(IF(OR(J19="",I19=0),"",J19/I19),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19="","",IF(J19&lt;=F19,"BAJO SEGURIDAD",IF(J19&lt;=G19,"PEDIR","OK")))</f>
+        <v/>
+      </c>
+      <c r="M19" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J6:J19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="El stock contado es un número mayor o igual a cero" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Trazabilidad: nombres completos en lugar de siglas
- Entradas y salidas: el día con su nombre completo y la fecha (Lunes 12/10) en lugar de L, M, M…
- Días de stock como «15 días»; seguridad y máximo sin abreviar; «Punto de pedido» y «Máximo» en
  las tablas; etapas del mapa de flujo con el nombre completo de cada control; «Insumos manuales,
  recargas y carros» en vez de «Ins.».
- Lugares del PT con el producto completo (Nuevo / Cilindro / Carro / Cilindro de carro / Sustituto).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Planilla_conteo_MP.xlsx
+++ b/salida/Planilla_conteo_MP.xlsx
@@ -14,12 +14,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Polvo" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embalaje" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identificación" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ins. manuales" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ins. recargas" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insumos manuales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insumos recargas" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soldadura" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gases" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casquetes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ins. carros" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insumos carros" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reventa (PT)" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
@@ -29,12 +29,12 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Polvo'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Embalaje'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Identificación'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Ins. manuales'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Ins. recargas'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Insumos manuales'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Insumos recargas'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'Soldadura'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'Gases'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'Casquetes'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="12">'Ins. carros'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'Insumos carros'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'Reventa (PT)'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>